<commit_message>
Implement analysis of TAM/UTAUT constructs in Streamlit app; update CSV outputs for open-ended questions and ranking metrics; enhance usability metrics and add new construct data.
</commit_message>
<xml_diff>
--- a/data/raw/Experiencia_en_el_uso_de_Power_App_B-Lab.xlsx
+++ b/data/raw/Experiencia_en_el_uso_de_Power_App_B-Lab.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David\Documents\Maestría en Estudios del Comportamiento\tablero_pre_pos_intervencion\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E139FA25-9E9C-452B-8ECF-789F2761A08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C8FB4F-9125-47B1-90BA-D87A34F07092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="-5460" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="114">
   <si>
     <t>Id</t>
   </si>
@@ -355,13 +355,25 @@
   </si>
   <si>
     <t>No, la veo práctica y de fácil consulta</t>
+  </si>
+  <si>
+    <t>llugo@bancolombia.com.co</t>
+  </si>
+  <si>
+    <t>Laura Isabel Lugo Perez</t>
+  </si>
+  <si>
+    <t>No tengo la solución, pero cuando intenté usarla, sentí que era más una herramienta de dcumentación. Puede ser porque normalmente estamos interactuando con otras plataformas donde las ciencias del comportamiento serían un atributo o parámetro incluido en un marco de trabajo general, no solo como un enfoque específico.</t>
+  </si>
+  <si>
+    <t>Lo dejé de usar por la misma razón de la respuesta anterior y porque el día a día de la iniciativa no nos permitió darle solo ese enfoque :(</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,6 +392,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -452,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -484,6 +503,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="22" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -766,8 +790,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -2353,6 +2381,62 @@
         <v>109</v>
       </c>
     </row>
+    <row r="30" spans="1:18" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="17">
+        <v>30</v>
+      </c>
+      <c r="B30" s="18">
+        <v>46118.493055555555</v>
+      </c>
+      <c r="C30" s="18">
+        <v>46118.495833333334</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H30" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="L30" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="M30" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="O30" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="P30" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q30" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="R30" s="19" t="s">
+        <v>113</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>